<commit_message>
EDA results: every family re-rendered with the coder-based PCT, plus the replicate report
Also catches up 9b9567f (MIPROC in QUESTIONNAIRE_ORDER) in families last rendered 2026-08-25/26:
MIPROC rows and figures appear, and MIPROC joins the compare_two_models / iso_compute Holm families
there (see history/CHANGELOG_EDA.md; open design question). No paper number comes from those
families. The replicate draws now carry the coder (384 calls on 2026-10-06).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Exp3_PTO_GRPO/eda/results/arms/heterogeneity/tables/claude-haiku-4-5/heterogeneity.xlsx
+++ b/Exp3_PTO_GRPO/eda/results/arms/heterogeneity/tables/claude-haiku-4-5/heterogeneity.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K217"/>
+  <dimension ref="A1:K241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5662,19 +5662,19 @@
         <v>32</v>
       </c>
       <c r="G122" t="n">
-        <v>0.9923177083333333</v>
+        <v>1</v>
       </c>
       <c r="H122" t="n">
-        <v>0.02473219860071983</v>
+        <v>0</v>
       </c>
       <c r="I122" t="n">
-        <v>0.004372076336055359</v>
+        <v>0</v>
       </c>
       <c r="J122" t="n">
-        <v>0.9318088755177572</v>
+        <v>0.9924107142857143</v>
       </c>
       <c r="K122" t="n">
-        <v>0.06050883281557617</v>
+        <v>0.007589285714285743</v>
       </c>
     </row>
     <row r="123">
@@ -5705,19 +5705,19 @@
         <v>32</v>
       </c>
       <c r="G123" t="n">
-        <v>0.2910428022270127</v>
+        <v>0.1730353956882489</v>
       </c>
       <c r="H123" t="n">
-        <v>0.1661655654009129</v>
+        <v>0.1924754610485592</v>
       </c>
       <c r="I123" t="n">
-        <v>0.02937419952367057</v>
+        <v>0.03402517592986085</v>
       </c>
       <c r="J123" t="n">
-        <v>0.1693683830247466</v>
+        <v>0.08357197831328982</v>
       </c>
       <c r="K123" t="n">
-        <v>0.1216744192022662</v>
+        <v>0.08946341737495912</v>
       </c>
     </row>
     <row r="124">
@@ -5748,19 +5748,19 @@
         <v>32</v>
       </c>
       <c r="G124" t="n">
-        <v>0.5541294642857142</v>
+        <v>0.567907370030332</v>
       </c>
       <c r="H124" t="n">
-        <v>0.1523349783121244</v>
+        <v>0.1687808523615688</v>
       </c>
       <c r="I124" t="n">
-        <v>0.0269292740441022</v>
+        <v>0.02983652130982771</v>
       </c>
       <c r="J124" t="n">
-        <v>0.4760499418662319</v>
+        <v>0.49312834433079</v>
       </c>
       <c r="K124" t="n">
-        <v>0.07807952241948229</v>
+        <v>0.07477902569954198</v>
       </c>
     </row>
     <row r="125">
@@ -5791,19 +5791,19 @@
         <v>32</v>
       </c>
       <c r="G125" t="n">
-        <v>0.961842411061161</v>
+        <v>0.9892857142857143</v>
       </c>
       <c r="H125" t="n">
-        <v>0.05802440130576771</v>
+        <v>0.04278026899640618</v>
       </c>
       <c r="I125" t="n">
-        <v>0.01025736190939948</v>
+        <v>0.007562554577085856</v>
       </c>
       <c r="J125" t="n">
-        <v>0.9318088755177572</v>
+        <v>0.9924107142857143</v>
       </c>
       <c r="K125" t="n">
-        <v>0.03003353554340382</v>
+        <v>-0.003124999999999933</v>
       </c>
     </row>
     <row r="126">
@@ -5834,19 +5834,19 @@
         <v>32</v>
       </c>
       <c r="G126" t="n">
-        <v>0.2445720308841186</v>
+        <v>0.1778874209671907</v>
       </c>
       <c r="H126" t="n">
-        <v>0.1563618061652371</v>
+        <v>0.2052905825238733</v>
       </c>
       <c r="I126" t="n">
-        <v>0.02764112336450392</v>
+        <v>0.03629059075409184</v>
       </c>
       <c r="J126" t="n">
-        <v>0.1693683830247466</v>
+        <v>0.08357197831328982</v>
       </c>
       <c r="K126" t="n">
-        <v>0.07520364785937203</v>
+        <v>0.09431544265390089</v>
       </c>
     </row>
     <row r="127">
@@ -5874,22 +5874,22 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G127" t="n">
-        <v>0.595475480401951</v>
+        <v>0.6407139325270754</v>
       </c>
       <c r="H127" t="n">
-        <v>0.139476087644177</v>
+        <v>0.1140751446274194</v>
       </c>
       <c r="I127" t="n">
-        <v>0.02465612184664169</v>
+        <v>0.02048850080455569</v>
       </c>
       <c r="J127" t="n">
-        <v>0.4760499418662319</v>
+        <v>0.49312834433079</v>
       </c>
       <c r="K127" t="n">
-        <v>0.1194255385357191</v>
+        <v>0.1475855881962854</v>
       </c>
     </row>
     <row r="128">
@@ -5920,19 +5920,19 @@
         <v>32</v>
       </c>
       <c r="G128" t="n">
-        <v>0.9889993686868688</v>
+        <v>0.9948958333333333</v>
       </c>
       <c r="H128" t="n">
-        <v>0.03071077218021904</v>
+        <v>0.01733052861923786</v>
       </c>
       <c r="I128" t="n">
-        <v>0.005428948816027014</v>
+        <v>0.003063633577052656</v>
       </c>
       <c r="J128" t="n">
-        <v>0.9450247975064152</v>
+        <v>0.9336630949728376</v>
       </c>
       <c r="K128" t="n">
-        <v>0.04397457118045356</v>
+        <v>0.0612327383604957</v>
       </c>
     </row>
     <row r="129">
@@ -5963,19 +5963,19 @@
         <v>32</v>
       </c>
       <c r="G129" t="n">
-        <v>0.4130962011307406</v>
+        <v>0.4413267309302064</v>
       </c>
       <c r="H129" t="n">
-        <v>0.2020150138961032</v>
+        <v>0.2936915401206614</v>
       </c>
       <c r="I129" t="n">
-        <v>0.0357115465568573</v>
+        <v>0.05191781989911017</v>
       </c>
       <c r="J129" t="n">
-        <v>0.1474739774829163</v>
+        <v>0.05229853887942123</v>
       </c>
       <c r="K129" t="n">
-        <v>0.2656222236478243</v>
+        <v>0.3890281920507851</v>
       </c>
     </row>
     <row r="130">
@@ -6006,19 +6006,19 @@
         <v>32</v>
       </c>
       <c r="G130" t="n">
-        <v>0.7735815011925209</v>
+        <v>0.7763007305194805</v>
       </c>
       <c r="H130" t="n">
-        <v>0.09624511268276728</v>
+        <v>0.1014230597029597</v>
       </c>
       <c r="I130" t="n">
-        <v>0.01701389295851203</v>
+        <v>0.01792923332116272</v>
       </c>
       <c r="J130" t="n">
-        <v>0.4271739153255529</v>
+        <v>0.4456312824803074</v>
       </c>
       <c r="K130" t="n">
-        <v>0.346407585866968</v>
+        <v>0.330669448039173</v>
       </c>
     </row>
     <row r="131">
@@ -6049,19 +6049,19 @@
         <v>32</v>
       </c>
       <c r="G131" t="n">
-        <v>0.9627232142857143</v>
+        <v>0.9965277777777778</v>
       </c>
       <c r="H131" t="n">
-        <v>0.05903906884914606</v>
+        <v>0.01964185503295966</v>
       </c>
       <c r="I131" t="n">
-        <v>0.01043673148454266</v>
+        <v>0.003472222222222223</v>
       </c>
       <c r="J131" t="n">
-        <v>0.9450247975064152</v>
+        <v>0.9336630949728376</v>
       </c>
       <c r="K131" t="n">
-        <v>0.01769841677929906</v>
+        <v>0.06286468280494018</v>
       </c>
     </row>
     <row r="132">
@@ -6092,19 +6092,19 @@
         <v>32</v>
       </c>
       <c r="G132" t="n">
-        <v>0.2814641990169273</v>
+        <v>0.2599873161100278</v>
       </c>
       <c r="H132" t="n">
-        <v>0.1846698310379603</v>
+        <v>0.2713158615818145</v>
       </c>
       <c r="I132" t="n">
-        <v>0.03264532245187893</v>
+        <v>0.04796232139199293</v>
       </c>
       <c r="J132" t="n">
-        <v>0.1474739774829163</v>
+        <v>0.05229853887942123</v>
       </c>
       <c r="K132" t="n">
-        <v>0.1339902215340111</v>
+        <v>0.2076887772306066</v>
       </c>
     </row>
     <row r="133">
@@ -6135,19 +6135,19 @@
         <v>32</v>
       </c>
       <c r="G133" t="n">
-        <v>0.7596610032876481</v>
+        <v>0.7705831299230899</v>
       </c>
       <c r="H133" t="n">
-        <v>0.08549914672634747</v>
+        <v>0.1083789188362696</v>
       </c>
       <c r="I133" t="n">
-        <v>0.01511425660896597</v>
+        <v>0.01915886711169816</v>
       </c>
       <c r="J133" t="n">
-        <v>0.4271739153255529</v>
+        <v>0.4456312824803074</v>
       </c>
       <c r="K133" t="n">
-        <v>0.3324870879620952</v>
+        <v>0.3249518474427824</v>
       </c>
     </row>
     <row r="134">
@@ -6178,19 +6178,19 @@
         <v>32</v>
       </c>
       <c r="G134" t="n">
-        <v>0.975483630952381</v>
+        <v>0.9934895833333333</v>
       </c>
       <c r="H134" t="n">
-        <v>0.05261769167769378</v>
+        <v>0.02615900982076477</v>
       </c>
       <c r="I134" t="n">
-        <v>0.009301581648920058</v>
+        <v>0.004624303308347065</v>
       </c>
       <c r="J134" t="n">
-        <v>0.9442857261525025</v>
+        <v>0.9848800505050506</v>
       </c>
       <c r="K134" t="n">
-        <v>0.0311979047998785</v>
+        <v>0.008609532828282696</v>
       </c>
     </row>
     <row r="135">
@@ -6221,19 +6221,19 @@
         <v>32</v>
       </c>
       <c r="G135" t="n">
-        <v>0.3451776522089022</v>
+        <v>0.2788797094718147</v>
       </c>
       <c r="H135" t="n">
-        <v>0.1254231246282574</v>
+        <v>0.1720965507415233</v>
       </c>
       <c r="I135" t="n">
-        <v>0.02217188548556157</v>
+        <v>0.03042265951203648</v>
       </c>
       <c r="J135" t="n">
-        <v>0.1951641021893054</v>
+        <v>0.08210403148310126</v>
       </c>
       <c r="K135" t="n">
-        <v>0.1500135500195968</v>
+        <v>0.1967756779887135</v>
       </c>
     </row>
     <row r="136">
@@ -6264,19 +6264,19 @@
         <v>32</v>
       </c>
       <c r="G136" t="n">
-        <v>0.5789558531746031</v>
+        <v>0.5679481976356977</v>
       </c>
       <c r="H136" t="n">
-        <v>0.182183653006762</v>
+        <v>0.1755480781190479</v>
       </c>
       <c r="I136" t="n">
-        <v>0.0322058241156046</v>
+        <v>0.03103280911556114</v>
       </c>
       <c r="J136" t="n">
-        <v>0.4201038499147052</v>
+        <v>0.4381522119740045</v>
       </c>
       <c r="K136" t="n">
-        <v>0.1588520032598979</v>
+        <v>0.1297959856616932</v>
       </c>
     </row>
     <row r="137">
@@ -6307,19 +6307,19 @@
         <v>32</v>
       </c>
       <c r="G137" t="n">
-        <v>0.9645337301587301</v>
+        <v>0.9916294642857143</v>
       </c>
       <c r="H137" t="n">
-        <v>0.06281592023792029</v>
+        <v>0.03301566367488849</v>
       </c>
       <c r="I137" t="n">
-        <v>0.01110439079167668</v>
+        <v>0.005836399917472005</v>
       </c>
       <c r="J137" t="n">
-        <v>0.9442857261525025</v>
+        <v>0.9848800505050506</v>
       </c>
       <c r="K137" t="n">
-        <v>0.02024800400622762</v>
+        <v>0.006749413780663738</v>
       </c>
     </row>
     <row r="138">
@@ -6347,22 +6347,22 @@
         </is>
       </c>
       <c r="F138" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G138" t="n">
-        <v>0.3210108493426508</v>
+        <v>0.2557676241886768</v>
       </c>
       <c r="H138" t="n">
-        <v>0.1806200983329109</v>
+        <v>0.2129611862896624</v>
       </c>
       <c r="I138" t="n">
-        <v>0.03192942408744558</v>
+        <v>0.03888121520130267</v>
       </c>
       <c r="J138" t="n">
-        <v>0.1951641021893054</v>
+        <v>0.08210403148310126</v>
       </c>
       <c r="K138" t="n">
-        <v>0.1258467471533454</v>
+        <v>0.1736635927055756</v>
       </c>
     </row>
     <row r="139">
@@ -6393,19 +6393,19 @@
         <v>32</v>
       </c>
       <c r="G139" t="n">
-        <v>0.6281092171717172</v>
+        <v>0.6328170093795094</v>
       </c>
       <c r="H139" t="n">
-        <v>0.1011159239122472</v>
+        <v>0.102222977283414</v>
       </c>
       <c r="I139" t="n">
-        <v>0.01787493887107325</v>
+        <v>0.01807064010754511</v>
       </c>
       <c r="J139" t="n">
-        <v>0.4201038499147052</v>
+        <v>0.4381522119740045</v>
       </c>
       <c r="K139" t="n">
-        <v>0.208005367257012</v>
+        <v>0.1946647974055049</v>
       </c>
     </row>
     <row r="140">
@@ -6436,19 +6436,19 @@
         <v>32</v>
       </c>
       <c r="G140" t="n">
-        <v>0.9728778467908903</v>
+        <v>0.9975000000000001</v>
       </c>
       <c r="H140" t="n">
-        <v>0.05403318550596819</v>
+        <v>0.009837387536759303</v>
       </c>
       <c r="I140" t="n">
-        <v>0.009551807970095194</v>
+        <v>0.001739020859100632</v>
       </c>
       <c r="J140" t="n">
-        <v>0.9378666975873657</v>
+        <v>0.9642850758009154</v>
       </c>
       <c r="K140" t="n">
-        <v>0.03501114920352455</v>
+        <v>0.03321492419908467</v>
       </c>
     </row>
     <row r="141">
@@ -6479,19 +6479,19 @@
         <v>32</v>
       </c>
       <c r="G141" t="n">
-        <v>0.3978133885593251</v>
+        <v>0.3762265975929385</v>
       </c>
       <c r="H141" t="n">
-        <v>0.2212640465818749</v>
+        <v>0.2511010805367427</v>
       </c>
       <c r="I141" t="n">
-        <v>0.03911432694270497</v>
+        <v>0.04438881920270005</v>
       </c>
       <c r="J141" t="n">
-        <v>0.1842579295704296</v>
+        <v>0.0721388754863987</v>
       </c>
       <c r="K141" t="n">
-        <v>0.2135554589888956</v>
+        <v>0.3040877221065398</v>
       </c>
     </row>
     <row r="142">
@@ -6522,19 +6522,19 @@
         <v>32</v>
       </c>
       <c r="G142" t="n">
-        <v>0.6829657321844822</v>
+        <v>0.6654172874715154</v>
       </c>
       <c r="H142" t="n">
-        <v>0.1953181436245332</v>
+        <v>0.2036144656539708</v>
       </c>
       <c r="I142" t="n">
-        <v>0.03452769596141887</v>
+        <v>0.03599429235289953</v>
       </c>
       <c r="J142" t="n">
-        <v>0.4472909902597403</v>
+        <v>0.4639555655911743</v>
       </c>
       <c r="K142" t="n">
-        <v>0.2356747419247419</v>
+        <v>0.2014617218803411</v>
       </c>
     </row>
     <row r="143">
@@ -6565,19 +6565,19 @@
         <v>32</v>
       </c>
       <c r="G143" t="n">
-        <v>0.9625</v>
+        <v>0.9881572420634921</v>
       </c>
       <c r="H143" t="n">
-        <v>0.05915743192778</v>
+        <v>0.0376275520966137</v>
       </c>
       <c r="I143" t="n">
-        <v>0.0104576553184287</v>
+        <v>0.00665167431174141</v>
       </c>
       <c r="J143" t="n">
-        <v>0.9378666975873657</v>
+        <v>0.9642850758009154</v>
       </c>
       <c r="K143" t="n">
-        <v>0.02463330241263428</v>
+        <v>0.02387216626257671</v>
       </c>
     </row>
     <row r="144">
@@ -6605,22 +6605,22 @@
         </is>
       </c>
       <c r="F144" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G144" t="n">
-        <v>0.2810101561020678</v>
+        <v>0.2219754249545521</v>
       </c>
       <c r="H144" t="n">
-        <v>0.2267376669049994</v>
+        <v>0.2366548023703067</v>
       </c>
       <c r="I144" t="n">
-        <v>0.04008193545473542</v>
+        <v>0.04250445725580566</v>
       </c>
       <c r="J144" t="n">
-        <v>0.1842579295704296</v>
+        <v>0.0721388754863987</v>
       </c>
       <c r="K144" t="n">
-        <v>0.09675222653163826</v>
+        <v>0.1498365494681534</v>
       </c>
     </row>
     <row r="145">
@@ -6651,19 +6651,19 @@
         <v>32</v>
       </c>
       <c r="G145" t="n">
-        <v>0.5949165417915419</v>
+        <v>0.5691900762281197</v>
       </c>
       <c r="H145" t="n">
-        <v>0.2455356327060242</v>
+        <v>0.2458576106400791</v>
       </c>
       <c r="I145" t="n">
-        <v>0.04340497772733978</v>
+        <v>0.04346189592248045</v>
       </c>
       <c r="J145" t="n">
-        <v>0.4472909902597403</v>
+        <v>0.4639555655911743</v>
       </c>
       <c r="K145" t="n">
-        <v>0.1476255515318016</v>
+        <v>0.1052345106369453</v>
       </c>
     </row>
     <row r="146">
@@ -9760,6 +9760,1038 @@
       </c>
       <c r="K217" t="n">
         <v>0.8878676470588234</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>GRPO_LA0</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>10</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F218" t="n">
+        <v>32</v>
+      </c>
+      <c r="G218" t="n">
+        <v>0.03125</v>
+      </c>
+      <c r="H218" t="n">
+        <v>0.1767766952966369</v>
+      </c>
+      <c r="I218" t="n">
+        <v>0.03125</v>
+      </c>
+      <c r="J218" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K218" t="n">
+        <v>-0.21875</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>GRPO_LA0</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>10</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F219" t="n">
+        <v>32</v>
+      </c>
+      <c r="G219" t="n">
+        <v>0.28125</v>
+      </c>
+      <c r="H219" t="n">
+        <v>0.4568034093991744</v>
+      </c>
+      <c r="I219" t="n">
+        <v>0.08075219711382271</v>
+      </c>
+      <c r="J219" t="n">
+        <v>0.2351190476190476</v>
+      </c>
+      <c r="K219" t="n">
+        <v>0.04613095238095238</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>GRPO_LA0</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>10</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>StartLowAndChangesToHigh</t>
+        </is>
+      </c>
+      <c r="F220" t="n">
+        <v>32</v>
+      </c>
+      <c r="G220" t="n">
+        <v>0.21875</v>
+      </c>
+      <c r="H220" t="n">
+        <v>0.4200134406451544</v>
+      </c>
+      <c r="I220" t="n">
+        <v>0.07424858801742054</v>
+      </c>
+      <c r="J220" t="n">
+        <v>0.2375</v>
+      </c>
+      <c r="K220" t="n">
+        <v>-0.01874999999999999</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>GRPO_LA0</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>3</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F221" t="n">
+        <v>32</v>
+      </c>
+      <c r="G221" t="n">
+        <v>0.15625</v>
+      </c>
+      <c r="H221" t="n">
+        <v>0.3689020326284735</v>
+      </c>
+      <c r="I221" t="n">
+        <v>0.06521328221627366</v>
+      </c>
+      <c r="J221" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K221" t="n">
+        <v>-0.09375</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>GRPO_LA0</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>3</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F222" t="n">
+        <v>32</v>
+      </c>
+      <c r="G222" t="n">
+        <v>0.40625</v>
+      </c>
+      <c r="H222" t="n">
+        <v>0.4825587044348142</v>
+      </c>
+      <c r="I222" t="n">
+        <v>0.08530513305661301</v>
+      </c>
+      <c r="J222" t="n">
+        <v>0.2351190476190476</v>
+      </c>
+      <c r="K222" t="n">
+        <v>0.1711309523809524</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>GRPO_LA0</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>3</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>StartLowAndChangesToHigh</t>
+        </is>
+      </c>
+      <c r="F223" t="n">
+        <v>32</v>
+      </c>
+      <c r="G223" t="n">
+        <v>0.2916666666666666</v>
+      </c>
+      <c r="H223" t="n">
+        <v>0.4539748781200978</v>
+      </c>
+      <c r="I223" t="n">
+        <v>0.08025217870176439</v>
+      </c>
+      <c r="J223" t="n">
+        <v>0.2375</v>
+      </c>
+      <c r="K223" t="n">
+        <v>0.05416666666666664</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>GRPO_LA5</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>10</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F224" t="n">
+        <v>32</v>
+      </c>
+      <c r="G224" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H224" t="n">
+        <v>0.4399413450640599</v>
+      </c>
+      <c r="I224" t="n">
+        <v>0.07777137710478188</v>
+      </c>
+      <c r="J224" t="n">
+        <v>0.15625</v>
+      </c>
+      <c r="K224" t="n">
+        <v>0.59375</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>GRPO_LA5</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>10</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F225" t="n">
+        <v>32</v>
+      </c>
+      <c r="G225" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H225" t="n">
+        <v>0.4399413450640599</v>
+      </c>
+      <c r="I225" t="n">
+        <v>0.07777137710478188</v>
+      </c>
+      <c r="J225" t="n">
+        <v>0.1875</v>
+      </c>
+      <c r="K225" t="n">
+        <v>0.5625</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>GRPO_LA5</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>10</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>StartLowAndChangesToHigh</t>
+        </is>
+      </c>
+      <c r="F226" t="n">
+        <v>32</v>
+      </c>
+      <c r="G226" t="n">
+        <v>0.90625</v>
+      </c>
+      <c r="H226" t="n">
+        <v>0.2961445810802991</v>
+      </c>
+      <c r="I226" t="n">
+        <v>0.0523514603733822</v>
+      </c>
+      <c r="J226" t="n">
+        <v>0.2489583333333333</v>
+      </c>
+      <c r="K226" t="n">
+        <v>0.6572916666666666</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>GRPO_LA5</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>7</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F227" t="n">
+        <v>32</v>
+      </c>
+      <c r="G227" t="n">
+        <v>0.59375</v>
+      </c>
+      <c r="H227" t="n">
+        <v>0.498990917235846</v>
+      </c>
+      <c r="I227" t="n">
+        <v>0.08820996533199051</v>
+      </c>
+      <c r="J227" t="n">
+        <v>0.15625</v>
+      </c>
+      <c r="K227" t="n">
+        <v>0.4375</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>GRPO_LA5</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>7</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F228" t="n">
+        <v>32</v>
+      </c>
+      <c r="G228" t="n">
+        <v>0.59375</v>
+      </c>
+      <c r="H228" t="n">
+        <v>0.498990917235846</v>
+      </c>
+      <c r="I228" t="n">
+        <v>0.08820996533199051</v>
+      </c>
+      <c r="J228" t="n">
+        <v>0.1875</v>
+      </c>
+      <c r="K228" t="n">
+        <v>0.40625</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>GRPO_LA5</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>7</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>StartLowAndChangesToHigh</t>
+        </is>
+      </c>
+      <c r="F229" t="n">
+        <v>32</v>
+      </c>
+      <c r="G229" t="n">
+        <v>0.6875</v>
+      </c>
+      <c r="H229" t="n">
+        <v>0.4709290748598849</v>
+      </c>
+      <c r="I229" t="n">
+        <v>0.08324928557283298</v>
+      </c>
+      <c r="J229" t="n">
+        <v>0.2489583333333333</v>
+      </c>
+      <c r="K229" t="n">
+        <v>0.4385416666666667</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>PTO_LA0</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>10</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F230" t="n">
+        <v>32</v>
+      </c>
+      <c r="G230" t="n">
+        <v>0.09375</v>
+      </c>
+      <c r="H230" t="n">
+        <v>0.2961445810802991</v>
+      </c>
+      <c r="I230" t="n">
+        <v>0.0523514603733822</v>
+      </c>
+      <c r="J230" t="n">
+        <v>0.1875</v>
+      </c>
+      <c r="K230" t="n">
+        <v>-0.09375</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>PTO_LA0</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>10</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F231" t="n">
+        <v>32</v>
+      </c>
+      <c r="G231" t="n">
+        <v>0.390625</v>
+      </c>
+      <c r="H231" t="n">
+        <v>0.4725614162357051</v>
+      </c>
+      <c r="I231" t="n">
+        <v>0.08353784548684644</v>
+      </c>
+      <c r="J231" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K231" t="n">
+        <v>0.140625</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>PTO_LA0</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>10</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>StartLowAndChangesToHigh</t>
+        </is>
+      </c>
+      <c r="F232" t="n">
+        <v>32</v>
+      </c>
+      <c r="G232" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="H232" t="n">
+        <v>0.4709290748598849</v>
+      </c>
+      <c r="I232" t="n">
+        <v>0.08324928557283298</v>
+      </c>
+      <c r="J232" t="n">
+        <v>0.1875</v>
+      </c>
+      <c r="K232" t="n">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>PTO_LA0</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>9</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F233" t="n">
+        <v>32</v>
+      </c>
+      <c r="G233" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="H233" t="n">
+        <v>0.2459346884189824</v>
+      </c>
+      <c r="I233" t="n">
+        <v>0.04347552147751577</v>
+      </c>
+      <c r="J233" t="n">
+        <v>0.1875</v>
+      </c>
+      <c r="K233" t="n">
+        <v>-0.125</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>PTO_LA0</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>9</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F234" t="n">
+        <v>32</v>
+      </c>
+      <c r="G234" t="n">
+        <v>0.34375</v>
+      </c>
+      <c r="H234" t="n">
+        <v>0.4825587044348142</v>
+      </c>
+      <c r="I234" t="n">
+        <v>0.08530513305661301</v>
+      </c>
+      <c r="J234" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K234" t="n">
+        <v>0.09375</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>PTO_LA0</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>9</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>StartLowAndChangesToHigh</t>
+        </is>
+      </c>
+      <c r="F235" t="n">
+        <v>32</v>
+      </c>
+      <c r="G235" t="n">
+        <v>0.21875</v>
+      </c>
+      <c r="H235" t="n">
+        <v>0.4200134406451544</v>
+      </c>
+      <c r="I235" t="n">
+        <v>0.07424858801742054</v>
+      </c>
+      <c r="J235" t="n">
+        <v>0.1875</v>
+      </c>
+      <c r="K235" t="n">
+        <v>0.03125</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>PTO_LA5</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>10</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F236" t="n">
+        <v>32</v>
+      </c>
+      <c r="G236" t="n">
+        <v>0.34375</v>
+      </c>
+      <c r="H236" t="n">
+        <v>0.4825587044348142</v>
+      </c>
+      <c r="I236" t="n">
+        <v>0.08530513305661301</v>
+      </c>
+      <c r="J236" t="n">
+        <v>0.1875</v>
+      </c>
+      <c r="K236" t="n">
+        <v>0.15625</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>PTO_LA5</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>10</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F237" t="n">
+        <v>32</v>
+      </c>
+      <c r="G237" t="n">
+        <v>0.546875</v>
+      </c>
+      <c r="H237" t="n">
+        <v>0.4977266868861963</v>
+      </c>
+      <c r="I237" t="n">
+        <v>0.08798647886868571</v>
+      </c>
+      <c r="J237" t="n">
+        <v>0.203125</v>
+      </c>
+      <c r="K237" t="n">
+        <v>0.34375</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>PTO_LA5</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>10</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>StartLowAndChangesToHigh</t>
+        </is>
+      </c>
+      <c r="F238" t="n">
+        <v>32</v>
+      </c>
+      <c r="G238" t="n">
+        <v>0.4375</v>
+      </c>
+      <c r="H238" t="n">
+        <v>0.5040161287741853</v>
+      </c>
+      <c r="I238" t="n">
+        <v>0.08909830562090465</v>
+      </c>
+      <c r="J238" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="K238" t="n">
+        <v>0.2625</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>PTO_LA5</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>7</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F239" t="n">
+        <v>32</v>
+      </c>
+      <c r="G239" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="H239" t="n">
+        <v>0.4918693768379647</v>
+      </c>
+      <c r="I239" t="n">
+        <v>0.08695104295503155</v>
+      </c>
+      <c r="J239" t="n">
+        <v>0.1875</v>
+      </c>
+      <c r="K239" t="n">
+        <v>0.1875</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>PTO_LA5</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>7</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F240" t="n">
+        <v>32</v>
+      </c>
+      <c r="G240" t="n">
+        <v>0.265625</v>
+      </c>
+      <c r="H240" t="n">
+        <v>0.4396548316210592</v>
+      </c>
+      <c r="I240" t="n">
+        <v>0.07772072820517018</v>
+      </c>
+      <c r="J240" t="n">
+        <v>0.203125</v>
+      </c>
+      <c r="K240" t="n">
+        <v>0.0625</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>PTO_LA5</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>7</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>StartLowAndChangesToHigh</t>
+        </is>
+      </c>
+      <c r="F241" t="n">
+        <v>32</v>
+      </c>
+      <c r="G241" t="n">
+        <v>0.15625</v>
+      </c>
+      <c r="H241" t="n">
+        <v>0.3689020326284735</v>
+      </c>
+      <c r="I241" t="n">
+        <v>0.06521328221627366</v>
+      </c>
+      <c r="J241" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="K241" t="n">
+        <v>-0.01874999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -9773,7 +10805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K145"/>
+  <dimension ref="A1:K161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13301,19 +14333,19 @@
         <v>48</v>
       </c>
       <c r="G82" t="n">
-        <v>0.6184024567659435</v>
+        <v>0.595381401006401</v>
       </c>
       <c r="H82" t="n">
-        <v>0.3163946351106552</v>
+        <v>0.3635381818795743</v>
       </c>
       <c r="I82" t="n">
-        <v>0.04566763193782256</v>
+        <v>0.05247221679221985</v>
       </c>
       <c r="J82" t="n">
-        <v>0.5301687567815243</v>
+        <v>0.5411728546847254</v>
       </c>
       <c r="K82" t="n">
-        <v>0.08823369998441921</v>
+        <v>0.0542085463216756</v>
       </c>
     </row>
     <row r="83">
@@ -13344,19 +14376,19 @@
         <v>48</v>
       </c>
       <c r="G83" t="n">
-        <v>0.6065908597980966</v>
+        <v>0.565247109472653</v>
       </c>
       <c r="H83" t="n">
-        <v>0.3234812077283815</v>
+        <v>0.3788995509201062</v>
       </c>
       <c r="I83" t="n">
-        <v>0.04669049058994158</v>
+        <v>0.05468943942988792</v>
       </c>
       <c r="J83" t="n">
-        <v>0.5213160434909661</v>
+        <v>0.5049011699351373</v>
       </c>
       <c r="K83" t="n">
-        <v>0.08527481630713052</v>
+        <v>0.06034593953751566</v>
       </c>
     </row>
     <row r="84">
@@ -13387,19 +14419,19 @@
         <v>48</v>
       </c>
       <c r="G84" t="n">
-        <v>0.6057012245477634</v>
+        <v>0.6007985744010318</v>
       </c>
       <c r="H84" t="n">
-        <v>0.3107419840449335</v>
+        <v>0.3466152424337976</v>
       </c>
       <c r="I84" t="n">
-        <v>0.04485174203421519</v>
+        <v>0.05002960088109511</v>
       </c>
       <c r="J84" t="n">
-        <v>0.5301687567815243</v>
+        <v>0.5411728546847254</v>
       </c>
       <c r="K84" t="n">
-        <v>0.07553246776623912</v>
+        <v>0.05962571971630637</v>
       </c>
     </row>
     <row r="85">
@@ -13427,22 +14459,22 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G85" t="n">
-        <v>0.5955587236837236</v>
+        <v>0.6036880992592079</v>
       </c>
       <c r="H85" t="n">
-        <v>0.3312593654863659</v>
+        <v>0.3818932521814397</v>
       </c>
       <c r="I85" t="n">
-        <v>0.0478131709587845</v>
+        <v>0.05570485598254901</v>
       </c>
       <c r="J85" t="n">
-        <v>0.5213160434909661</v>
+        <v>0.5049011699351373</v>
       </c>
       <c r="K85" t="n">
-        <v>0.07424268019275759</v>
+        <v>0.09878692932407052</v>
       </c>
     </row>
     <row r="86">
@@ -13473,19 +14505,19 @@
         <v>48</v>
       </c>
       <c r="G86" t="n">
-        <v>0.7286242144794777</v>
+        <v>0.733671205902327</v>
       </c>
       <c r="H86" t="n">
-        <v>0.2546123530738583</v>
+        <v>0.2684953495401585</v>
       </c>
       <c r="I86" t="n">
-        <v>0.03675012764654904</v>
+        <v>0.03875396558329329</v>
       </c>
       <c r="J86" t="n">
-        <v>0.5110360802055091</v>
+        <v>0.4685884659322159</v>
       </c>
       <c r="K86" t="n">
-        <v>0.2175881342739686</v>
+        <v>0.2650827399701111</v>
       </c>
     </row>
     <row r="87">
@@ -13516,19 +14548,19 @@
         <v>48</v>
       </c>
       <c r="G87" t="n">
-        <v>0.7218271661939425</v>
+        <v>0.7413443239530194</v>
       </c>
       <c r="H87" t="n">
-        <v>0.2899881338960541</v>
+        <v>0.3124275702938965</v>
       </c>
       <c r="I87" t="n">
-        <v>0.04185618179167102</v>
+        <v>0.04509503545286046</v>
       </c>
       <c r="J87" t="n">
-        <v>0.5020790466710804</v>
+        <v>0.4858068116228282</v>
       </c>
       <c r="K87" t="n">
-        <v>0.2197481195228621</v>
+        <v>0.2555375123301912</v>
       </c>
     </row>
     <row r="88">
@@ -13559,19 +14591,19 @@
         <v>48</v>
       </c>
       <c r="G88" t="n">
-        <v>0.6694907842522975</v>
+        <v>0.6819643892741718</v>
       </c>
       <c r="H88" t="n">
-        <v>0.3167354434366582</v>
+        <v>0.3669369109868297</v>
       </c>
       <c r="I88" t="n">
-        <v>0.04571682338251253</v>
+        <v>0.05296278108346398</v>
       </c>
       <c r="J88" t="n">
-        <v>0.5110360802055091</v>
+        <v>0.4685884659322159</v>
       </c>
       <c r="K88" t="n">
-        <v>0.1584547040467884</v>
+        <v>0.2133759233419559</v>
       </c>
     </row>
     <row r="89">
@@ -13602,19 +14634,19 @@
         <v>48</v>
       </c>
       <c r="G89" t="n">
-        <v>0.6664081601412289</v>
+        <v>0.6694344265997584</v>
       </c>
       <c r="H89" t="n">
-        <v>0.3096352420157786</v>
+        <v>0.3401533398272007</v>
       </c>
       <c r="I89" t="n">
-        <v>0.04469199758210118</v>
+        <v>0.04909690557874614</v>
       </c>
       <c r="J89" t="n">
-        <v>0.5020790466710804</v>
+        <v>0.4858068116228282</v>
       </c>
       <c r="K89" t="n">
-        <v>0.1643291134701486</v>
+        <v>0.1836276149769301</v>
       </c>
     </row>
     <row r="90">
@@ -13645,19 +14677,19 @@
         <v>48</v>
       </c>
       <c r="G90" t="n">
-        <v>0.6458795833795834</v>
+        <v>0.6274445146929667</v>
       </c>
       <c r="H90" t="n">
-        <v>0.2853061467930575</v>
+        <v>0.3177641551765624</v>
       </c>
       <c r="I90" t="n">
-        <v>0.04118039516310667</v>
+        <v>0.04586530513250058</v>
       </c>
       <c r="J90" t="n">
-        <v>0.5134563311251585</v>
+        <v>0.4802608962400825</v>
       </c>
       <c r="K90" t="n">
-        <v>0.1324232522544249</v>
+        <v>0.1471836184528842</v>
       </c>
     </row>
     <row r="91">
@@ -13688,19 +14720,19 @@
         <v>48</v>
       </c>
       <c r="G91" t="n">
-        <v>0.6205318408443408</v>
+        <v>0.5994338122675971</v>
       </c>
       <c r="H91" t="n">
-        <v>0.3010280061082609</v>
+        <v>0.3389619867482621</v>
       </c>
       <c r="I91" t="n">
-        <v>0.04344965009005519</v>
+        <v>0.04892494857353986</v>
       </c>
       <c r="J91" t="n">
-        <v>0.5262461210458501</v>
+        <v>0.5249720462827879</v>
       </c>
       <c r="K91" t="n">
-        <v>0.09428571979849065</v>
+        <v>0.07446176598480914</v>
       </c>
     </row>
     <row r="92">
@@ -13728,22 +14760,22 @@
         </is>
       </c>
       <c r="F92" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G92" t="n">
-        <v>0.6359401032654709</v>
+        <v>0.644079185092623</v>
       </c>
       <c r="H92" t="n">
-        <v>0.3078406579959405</v>
+        <v>0.3344780660834215</v>
       </c>
       <c r="I92" t="n">
-        <v>0.04443297169036694</v>
+        <v>0.04878864026549049</v>
       </c>
       <c r="J92" t="n">
-        <v>0.5134563311251585</v>
+        <v>0.4802608962400825</v>
       </c>
       <c r="K92" t="n">
-        <v>0.1224837721403124</v>
+        <v>0.1638182888525405</v>
       </c>
     </row>
     <row r="93">
@@ -13771,22 +14803,22 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G93" t="n">
-        <v>0.6398290945165944</v>
+        <v>0.6251828549700889</v>
       </c>
       <c r="H93" t="n">
-        <v>0.2777870620755514</v>
+        <v>0.326471334285533</v>
       </c>
       <c r="I93" t="n">
-        <v>0.04009510876667872</v>
+        <v>0.04762073839986557</v>
       </c>
       <c r="J93" t="n">
-        <v>0.5262461210458501</v>
+        <v>0.5249720462827879</v>
       </c>
       <c r="K93" t="n">
-        <v>0.1135829734707443</v>
+        <v>0.1002108086873009</v>
       </c>
     </row>
     <row r="94">
@@ -13817,19 +14849,19 @@
         <v>48</v>
       </c>
       <c r="G94" t="n">
-        <v>0.7081757423862687</v>
+        <v>0.6921794602778543</v>
       </c>
       <c r="H94" t="n">
-        <v>0.2644502137272563</v>
+        <v>0.2890908000349903</v>
       </c>
       <c r="I94" t="n">
-        <v>0.03817010052067137</v>
+        <v>0.04172666280511148</v>
       </c>
       <c r="J94" t="n">
-        <v>0.506973581973582</v>
+        <v>0.5027280548300816</v>
       </c>
       <c r="K94" t="n">
-        <v>0.2012021604126867</v>
+        <v>0.1894514054477726</v>
       </c>
     </row>
     <row r="95">
@@ -13860,19 +14892,19 @@
         <v>48</v>
       </c>
       <c r="G95" t="n">
-        <v>0.660928902636863</v>
+        <v>0.6672497964317818</v>
       </c>
       <c r="H95" t="n">
-        <v>0.3176262129627035</v>
+        <v>0.3416312882209624</v>
       </c>
       <c r="I95" t="n">
-        <v>0.04584539488892458</v>
+        <v>0.04931022905449282</v>
       </c>
       <c r="J95" t="n">
-        <v>0.539303496304775</v>
+        <v>0.5157371960026594</v>
       </c>
       <c r="K95" t="n">
-        <v>0.121625406332088</v>
+        <v>0.1515126004291224</v>
       </c>
     </row>
     <row r="96">
@@ -13900,22 +14932,22 @@
         </is>
       </c>
       <c r="F96" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G96" t="n">
-        <v>0.6351327287908169</v>
+        <v>0.6206358150021425</v>
       </c>
       <c r="H96" t="n">
-        <v>0.3161186149058418</v>
+        <v>0.3509743040577748</v>
       </c>
       <c r="I96" t="n">
-        <v>0.04562779185293486</v>
+        <v>0.05119486387736678</v>
       </c>
       <c r="J96" t="n">
-        <v>0.506973581973582</v>
+        <v>0.5027280548300816</v>
       </c>
       <c r="K96" t="n">
-        <v>0.1281591468172349</v>
+        <v>0.1179077601720608</v>
       </c>
     </row>
     <row r="97">
@@ -13946,19 +14978,19 @@
         <v>48</v>
       </c>
       <c r="G97" t="n">
-        <v>0.5904850698049228</v>
+        <v>0.5738847719546248</v>
       </c>
       <c r="H97" t="n">
-        <v>0.3653252707626953</v>
+        <v>0.3903185599689186</v>
       </c>
       <c r="I97" t="n">
-        <v>0.05273016085415376</v>
+        <v>0.05633763141694056</v>
       </c>
       <c r="J97" t="n">
-        <v>0.539303496304775</v>
+        <v>0.5157371960026594</v>
       </c>
       <c r="K97" t="n">
-        <v>0.05118157350014774</v>
+        <v>0.0581475759519654</v>
       </c>
     </row>
     <row r="98">
@@ -16023,6 +17055,694 @@
       </c>
       <c r="K145" t="n">
         <v>0.7034313725490198</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>GRPO_LA0</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>10</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Obesity</t>
+        </is>
+      </c>
+      <c r="F146" t="n">
+        <v>48</v>
+      </c>
+      <c r="G146" t="n">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="H146" t="n">
+        <v>0.3766217885773548</v>
+      </c>
+      <c r="I146" t="n">
+        <v>0.05436067275445353</v>
+      </c>
+      <c r="J146" t="n">
+        <v>0.3150793650793651</v>
+      </c>
+      <c r="K146" t="n">
+        <v>-0.1484126984126984</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>GRPO_LA0</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>10</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Smoking</t>
+        </is>
+      </c>
+      <c r="F147" t="n">
+        <v>48</v>
+      </c>
+      <c r="G147" t="n">
+        <v>0.1875</v>
+      </c>
+      <c r="H147" t="n">
+        <v>0.3944427796055833</v>
+      </c>
+      <c r="I147" t="n">
+        <v>0.05693291124629694</v>
+      </c>
+      <c r="J147" t="n">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="K147" t="n">
+        <v>0.02083333333333334</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>GRPO_LA0</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>3</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Obesity</t>
+        </is>
+      </c>
+      <c r="F148" t="n">
+        <v>48</v>
+      </c>
+      <c r="G148" t="n">
+        <v>0.2986111111111111</v>
+      </c>
+      <c r="H148" t="n">
+        <v>0.4455696454031056</v>
+      </c>
+      <c r="I148" t="n">
+        <v>0.06431243867905229</v>
+      </c>
+      <c r="J148" t="n">
+        <v>0.3150793650793651</v>
+      </c>
+      <c r="K148" t="n">
+        <v>-0.01646825396825397</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>GRPO_LA0</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>3</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Smoking</t>
+        </is>
+      </c>
+      <c r="F149" t="n">
+        <v>48</v>
+      </c>
+      <c r="G149" t="n">
+        <v>0.2708333333333333</v>
+      </c>
+      <c r="H149" t="n">
+        <v>0.4490928602896294</v>
+      </c>
+      <c r="I149" t="n">
+        <v>0.06482097094483914</v>
+      </c>
+      <c r="J149" t="n">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="K149" t="n">
+        <v>0.1041666666666667</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>GRPO_LA5</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>10</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Obesity</t>
+        </is>
+      </c>
+      <c r="F150" t="n">
+        <v>48</v>
+      </c>
+      <c r="G150" t="n">
+        <v>0.8125</v>
+      </c>
+      <c r="H150" t="n">
+        <v>0.3944427796055833</v>
+      </c>
+      <c r="I150" t="n">
+        <v>0.05693291124629694</v>
+      </c>
+      <c r="J150" t="n">
+        <v>0.2597222222222222</v>
+      </c>
+      <c r="K150" t="n">
+        <v>0.5527777777777778</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>GRPO_LA5</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>10</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Smoking</t>
+        </is>
+      </c>
+      <c r="F151" t="n">
+        <v>48</v>
+      </c>
+      <c r="G151" t="n">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="H151" t="n">
+        <v>0.4104140790860576</v>
+      </c>
+      <c r="I151" t="n">
+        <v>0.05923816975988693</v>
+      </c>
+      <c r="J151" t="n">
+        <v>0.1354166666666667</v>
+      </c>
+      <c r="K151" t="n">
+        <v>0.65625</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>GRPO_LA5</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>7</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Obesity</t>
+        </is>
+      </c>
+      <c r="F152" t="n">
+        <v>48</v>
+      </c>
+      <c r="G152" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="H152" t="n">
+        <v>0.4892460547900817</v>
+      </c>
+      <c r="I152" t="n">
+        <v>0.07061658535825402</v>
+      </c>
+      <c r="J152" t="n">
+        <v>0.2597222222222222</v>
+      </c>
+      <c r="K152" t="n">
+        <v>0.3652777777777778</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>GRPO_LA5</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>7</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Smoking</t>
+        </is>
+      </c>
+      <c r="F153" t="n">
+        <v>48</v>
+      </c>
+      <c r="G153" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="H153" t="n">
+        <v>0.4892460547900817</v>
+      </c>
+      <c r="I153" t="n">
+        <v>0.07061658535825402</v>
+      </c>
+      <c r="J153" t="n">
+        <v>0.1354166666666667</v>
+      </c>
+      <c r="K153" t="n">
+        <v>0.4895833333333334</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>PTO_LA0</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>10</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Obesity</t>
+        </is>
+      </c>
+      <c r="F154" t="n">
+        <v>48</v>
+      </c>
+      <c r="G154" t="n">
+        <v>0.2291666666666667</v>
+      </c>
+      <c r="H154" t="n">
+        <v>0.4247443953937942</v>
+      </c>
+      <c r="I154" t="n">
+        <v>0.06130657275434798</v>
+      </c>
+      <c r="J154" t="n">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="K154" t="n">
+        <v>0.0625</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>PTO_LA0</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>10</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Smoking</t>
+        </is>
+      </c>
+      <c r="F155" t="n">
+        <v>48</v>
+      </c>
+      <c r="G155" t="n">
+        <v>0.3020833333333333</v>
+      </c>
+      <c r="H155" t="n">
+        <v>0.4478161482131621</v>
+      </c>
+      <c r="I155" t="n">
+        <v>0.06463669342958263</v>
+      </c>
+      <c r="J155" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K155" t="n">
+        <v>0.05208333333333331</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>PTO_LA0</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>9</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Obesity</t>
+        </is>
+      </c>
+      <c r="F156" t="n">
+        <v>48</v>
+      </c>
+      <c r="G156" t="n">
+        <v>0.2083333333333333</v>
+      </c>
+      <c r="H156" t="n">
+        <v>0.4104140790860576</v>
+      </c>
+      <c r="I156" t="n">
+        <v>0.05923816975988693</v>
+      </c>
+      <c r="J156" t="n">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="K156" t="n">
+        <v>0.04166666666666669</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>PTO_LA0</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>9</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Smoking</t>
+        </is>
+      </c>
+      <c r="F157" t="n">
+        <v>48</v>
+      </c>
+      <c r="G157" t="n">
+        <v>0.2083333333333333</v>
+      </c>
+      <c r="H157" t="n">
+        <v>0.4104140790860576</v>
+      </c>
+      <c r="I157" t="n">
+        <v>0.05923816975988693</v>
+      </c>
+      <c r="J157" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K157" t="n">
+        <v>-0.04166666666666666</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>PTO_LA5</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>10</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Obesity</t>
+        </is>
+      </c>
+      <c r="F158" t="n">
+        <v>48</v>
+      </c>
+      <c r="G158" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H158" t="n">
+        <v>0.5052911526399113</v>
+      </c>
+      <c r="I158" t="n">
+        <v>0.07293249574894728</v>
+      </c>
+      <c r="J158" t="n">
+        <v>0.1479166666666667</v>
+      </c>
+      <c r="K158" t="n">
+        <v>0.3520833333333333</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>PTO_LA5</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>10</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Smoking</t>
+        </is>
+      </c>
+      <c r="F159" t="n">
+        <v>48</v>
+      </c>
+      <c r="G159" t="n">
+        <v>0.3854166666666667</v>
+      </c>
+      <c r="H159" t="n">
+        <v>0.4864065296197591</v>
+      </c>
+      <c r="I159" t="n">
+        <v>0.07020673520288989</v>
+      </c>
+      <c r="J159" t="n">
+        <v>0.2291666666666667</v>
+      </c>
+      <c r="K159" t="n">
+        <v>0.15625</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>PTO_LA5</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>7</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Obesity</t>
+        </is>
+      </c>
+      <c r="F160" t="n">
+        <v>48</v>
+      </c>
+      <c r="G160" t="n">
+        <v>0.3645833333333333</v>
+      </c>
+      <c r="H160" t="n">
+        <v>0.480907645105136</v>
+      </c>
+      <c r="I160" t="n">
+        <v>0.06941303958919982</v>
+      </c>
+      <c r="J160" t="n">
+        <v>0.1479166666666667</v>
+      </c>
+      <c r="K160" t="n">
+        <v>0.2166666666666666</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>MIPROC</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>best</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>PTO_LA5</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>7</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Smoking</t>
+        </is>
+      </c>
+      <c r="F161" t="n">
+        <v>48</v>
+      </c>
+      <c r="G161" t="n">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="H161" t="n">
+        <v>0.3766217885773547</v>
+      </c>
+      <c r="I161" t="n">
+        <v>0.05436067275445352</v>
+      </c>
+      <c r="J161" t="n">
+        <v>0.2291666666666667</v>
+      </c>
+      <c r="K161" t="n">
+        <v>-0.0625</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EDA results: re-rendered with MIPROC out of the outcome corrections (arms, compute, method, lookahead, measurement)
The pooled judge-agreement ladder is back on the eight instruments (7,525 contrasts, 88.3%); the MIPROC
panels the 2026-10-06 render added to arms/* are gone again.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Exp3_PTO_GRPO/eda/results/arms/heterogeneity/tables/claude-haiku-4-5/heterogeneity.xlsx
+++ b/Exp3_PTO_GRPO/eda/results/arms/heterogeneity/tables/claude-haiku-4-5/heterogeneity.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K241"/>
+  <dimension ref="A1:K217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9760,1038 +9760,6 @@
       </c>
       <c r="K217" t="n">
         <v>0.8878676470588234</v>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B218" t="inlineStr">
-        <is>
-          <t>final</t>
-        </is>
-      </c>
-      <c r="C218" t="inlineStr">
-        <is>
-          <t>GRPO_LA0</t>
-        </is>
-      </c>
-      <c r="D218" t="n">
-        <v>10</v>
-      </c>
-      <c r="E218" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F218" t="n">
-        <v>32</v>
-      </c>
-      <c r="G218" t="n">
-        <v>0.03125</v>
-      </c>
-      <c r="H218" t="n">
-        <v>0.1767766952966369</v>
-      </c>
-      <c r="I218" t="n">
-        <v>0.03125</v>
-      </c>
-      <c r="J218" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="K218" t="n">
-        <v>-0.21875</v>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B219" t="inlineStr">
-        <is>
-          <t>final</t>
-        </is>
-      </c>
-      <c r="C219" t="inlineStr">
-        <is>
-          <t>GRPO_LA0</t>
-        </is>
-      </c>
-      <c r="D219" t="n">
-        <v>10</v>
-      </c>
-      <c r="E219" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F219" t="n">
-        <v>32</v>
-      </c>
-      <c r="G219" t="n">
-        <v>0.28125</v>
-      </c>
-      <c r="H219" t="n">
-        <v>0.4568034093991744</v>
-      </c>
-      <c r="I219" t="n">
-        <v>0.08075219711382271</v>
-      </c>
-      <c r="J219" t="n">
-        <v>0.2351190476190476</v>
-      </c>
-      <c r="K219" t="n">
-        <v>0.04613095238095238</v>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B220" t="inlineStr">
-        <is>
-          <t>final</t>
-        </is>
-      </c>
-      <c r="C220" t="inlineStr">
-        <is>
-          <t>GRPO_LA0</t>
-        </is>
-      </c>
-      <c r="D220" t="n">
-        <v>10</v>
-      </c>
-      <c r="E220" t="inlineStr">
-        <is>
-          <t>StartLowAndChangesToHigh</t>
-        </is>
-      </c>
-      <c r="F220" t="n">
-        <v>32</v>
-      </c>
-      <c r="G220" t="n">
-        <v>0.21875</v>
-      </c>
-      <c r="H220" t="n">
-        <v>0.4200134406451544</v>
-      </c>
-      <c r="I220" t="n">
-        <v>0.07424858801742054</v>
-      </c>
-      <c r="J220" t="n">
-        <v>0.2375</v>
-      </c>
-      <c r="K220" t="n">
-        <v>-0.01874999999999999</v>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B221" t="inlineStr">
-        <is>
-          <t>best</t>
-        </is>
-      </c>
-      <c r="C221" t="inlineStr">
-        <is>
-          <t>GRPO_LA0</t>
-        </is>
-      </c>
-      <c r="D221" t="n">
-        <v>3</v>
-      </c>
-      <c r="E221" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F221" t="n">
-        <v>32</v>
-      </c>
-      <c r="G221" t="n">
-        <v>0.15625</v>
-      </c>
-      <c r="H221" t="n">
-        <v>0.3689020326284735</v>
-      </c>
-      <c r="I221" t="n">
-        <v>0.06521328221627366</v>
-      </c>
-      <c r="J221" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="K221" t="n">
-        <v>-0.09375</v>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B222" t="inlineStr">
-        <is>
-          <t>best</t>
-        </is>
-      </c>
-      <c r="C222" t="inlineStr">
-        <is>
-          <t>GRPO_LA0</t>
-        </is>
-      </c>
-      <c r="D222" t="n">
-        <v>3</v>
-      </c>
-      <c r="E222" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F222" t="n">
-        <v>32</v>
-      </c>
-      <c r="G222" t="n">
-        <v>0.40625</v>
-      </c>
-      <c r="H222" t="n">
-        <v>0.4825587044348142</v>
-      </c>
-      <c r="I222" t="n">
-        <v>0.08530513305661301</v>
-      </c>
-      <c r="J222" t="n">
-        <v>0.2351190476190476</v>
-      </c>
-      <c r="K222" t="n">
-        <v>0.1711309523809524</v>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B223" t="inlineStr">
-        <is>
-          <t>best</t>
-        </is>
-      </c>
-      <c r="C223" t="inlineStr">
-        <is>
-          <t>GRPO_LA0</t>
-        </is>
-      </c>
-      <c r="D223" t="n">
-        <v>3</v>
-      </c>
-      <c r="E223" t="inlineStr">
-        <is>
-          <t>StartLowAndChangesToHigh</t>
-        </is>
-      </c>
-      <c r="F223" t="n">
-        <v>32</v>
-      </c>
-      <c r="G223" t="n">
-        <v>0.2916666666666666</v>
-      </c>
-      <c r="H223" t="n">
-        <v>0.4539748781200978</v>
-      </c>
-      <c r="I223" t="n">
-        <v>0.08025217870176439</v>
-      </c>
-      <c r="J223" t="n">
-        <v>0.2375</v>
-      </c>
-      <c r="K223" t="n">
-        <v>0.05416666666666664</v>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B224" t="inlineStr">
-        <is>
-          <t>final</t>
-        </is>
-      </c>
-      <c r="C224" t="inlineStr">
-        <is>
-          <t>GRPO_LA5</t>
-        </is>
-      </c>
-      <c r="D224" t="n">
-        <v>10</v>
-      </c>
-      <c r="E224" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F224" t="n">
-        <v>32</v>
-      </c>
-      <c r="G224" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="H224" t="n">
-        <v>0.4399413450640599</v>
-      </c>
-      <c r="I224" t="n">
-        <v>0.07777137710478188</v>
-      </c>
-      <c r="J224" t="n">
-        <v>0.15625</v>
-      </c>
-      <c r="K224" t="n">
-        <v>0.59375</v>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B225" t="inlineStr">
-        <is>
-          <t>final</t>
-        </is>
-      </c>
-      <c r="C225" t="inlineStr">
-        <is>
-          <t>GRPO_LA5</t>
-        </is>
-      </c>
-      <c r="D225" t="n">
-        <v>10</v>
-      </c>
-      <c r="E225" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F225" t="n">
-        <v>32</v>
-      </c>
-      <c r="G225" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="H225" t="n">
-        <v>0.4399413450640599</v>
-      </c>
-      <c r="I225" t="n">
-        <v>0.07777137710478188</v>
-      </c>
-      <c r="J225" t="n">
-        <v>0.1875</v>
-      </c>
-      <c r="K225" t="n">
-        <v>0.5625</v>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B226" t="inlineStr">
-        <is>
-          <t>final</t>
-        </is>
-      </c>
-      <c r="C226" t="inlineStr">
-        <is>
-          <t>GRPO_LA5</t>
-        </is>
-      </c>
-      <c r="D226" t="n">
-        <v>10</v>
-      </c>
-      <c r="E226" t="inlineStr">
-        <is>
-          <t>StartLowAndChangesToHigh</t>
-        </is>
-      </c>
-      <c r="F226" t="n">
-        <v>32</v>
-      </c>
-      <c r="G226" t="n">
-        <v>0.90625</v>
-      </c>
-      <c r="H226" t="n">
-        <v>0.2961445810802991</v>
-      </c>
-      <c r="I226" t="n">
-        <v>0.0523514603733822</v>
-      </c>
-      <c r="J226" t="n">
-        <v>0.2489583333333333</v>
-      </c>
-      <c r="K226" t="n">
-        <v>0.6572916666666666</v>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B227" t="inlineStr">
-        <is>
-          <t>best</t>
-        </is>
-      </c>
-      <c r="C227" t="inlineStr">
-        <is>
-          <t>GRPO_LA5</t>
-        </is>
-      </c>
-      <c r="D227" t="n">
-        <v>7</v>
-      </c>
-      <c r="E227" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F227" t="n">
-        <v>32</v>
-      </c>
-      <c r="G227" t="n">
-        <v>0.59375</v>
-      </c>
-      <c r="H227" t="n">
-        <v>0.498990917235846</v>
-      </c>
-      <c r="I227" t="n">
-        <v>0.08820996533199051</v>
-      </c>
-      <c r="J227" t="n">
-        <v>0.15625</v>
-      </c>
-      <c r="K227" t="n">
-        <v>0.4375</v>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B228" t="inlineStr">
-        <is>
-          <t>best</t>
-        </is>
-      </c>
-      <c r="C228" t="inlineStr">
-        <is>
-          <t>GRPO_LA5</t>
-        </is>
-      </c>
-      <c r="D228" t="n">
-        <v>7</v>
-      </c>
-      <c r="E228" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F228" t="n">
-        <v>32</v>
-      </c>
-      <c r="G228" t="n">
-        <v>0.59375</v>
-      </c>
-      <c r="H228" t="n">
-        <v>0.498990917235846</v>
-      </c>
-      <c r="I228" t="n">
-        <v>0.08820996533199051</v>
-      </c>
-      <c r="J228" t="n">
-        <v>0.1875</v>
-      </c>
-      <c r="K228" t="n">
-        <v>0.40625</v>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B229" t="inlineStr">
-        <is>
-          <t>best</t>
-        </is>
-      </c>
-      <c r="C229" t="inlineStr">
-        <is>
-          <t>GRPO_LA5</t>
-        </is>
-      </c>
-      <c r="D229" t="n">
-        <v>7</v>
-      </c>
-      <c r="E229" t="inlineStr">
-        <is>
-          <t>StartLowAndChangesToHigh</t>
-        </is>
-      </c>
-      <c r="F229" t="n">
-        <v>32</v>
-      </c>
-      <c r="G229" t="n">
-        <v>0.6875</v>
-      </c>
-      <c r="H229" t="n">
-        <v>0.4709290748598849</v>
-      </c>
-      <c r="I229" t="n">
-        <v>0.08324928557283298</v>
-      </c>
-      <c r="J229" t="n">
-        <v>0.2489583333333333</v>
-      </c>
-      <c r="K229" t="n">
-        <v>0.4385416666666667</v>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B230" t="inlineStr">
-        <is>
-          <t>final</t>
-        </is>
-      </c>
-      <c r="C230" t="inlineStr">
-        <is>
-          <t>PTO_LA0</t>
-        </is>
-      </c>
-      <c r="D230" t="n">
-        <v>10</v>
-      </c>
-      <c r="E230" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F230" t="n">
-        <v>32</v>
-      </c>
-      <c r="G230" t="n">
-        <v>0.09375</v>
-      </c>
-      <c r="H230" t="n">
-        <v>0.2961445810802991</v>
-      </c>
-      <c r="I230" t="n">
-        <v>0.0523514603733822</v>
-      </c>
-      <c r="J230" t="n">
-        <v>0.1875</v>
-      </c>
-      <c r="K230" t="n">
-        <v>-0.09375</v>
-      </c>
-    </row>
-    <row r="231">
-      <c r="A231" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B231" t="inlineStr">
-        <is>
-          <t>final</t>
-        </is>
-      </c>
-      <c r="C231" t="inlineStr">
-        <is>
-          <t>PTO_LA0</t>
-        </is>
-      </c>
-      <c r="D231" t="n">
-        <v>10</v>
-      </c>
-      <c r="E231" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F231" t="n">
-        <v>32</v>
-      </c>
-      <c r="G231" t="n">
-        <v>0.390625</v>
-      </c>
-      <c r="H231" t="n">
-        <v>0.4725614162357051</v>
-      </c>
-      <c r="I231" t="n">
-        <v>0.08353784548684644</v>
-      </c>
-      <c r="J231" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="K231" t="n">
-        <v>0.140625</v>
-      </c>
-    </row>
-    <row r="232">
-      <c r="A232" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B232" t="inlineStr">
-        <is>
-          <t>final</t>
-        </is>
-      </c>
-      <c r="C232" t="inlineStr">
-        <is>
-          <t>PTO_LA0</t>
-        </is>
-      </c>
-      <c r="D232" t="n">
-        <v>10</v>
-      </c>
-      <c r="E232" t="inlineStr">
-        <is>
-          <t>StartLowAndChangesToHigh</t>
-        </is>
-      </c>
-      <c r="F232" t="n">
-        <v>32</v>
-      </c>
-      <c r="G232" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="H232" t="n">
-        <v>0.4709290748598849</v>
-      </c>
-      <c r="I232" t="n">
-        <v>0.08324928557283298</v>
-      </c>
-      <c r="J232" t="n">
-        <v>0.1875</v>
-      </c>
-      <c r="K232" t="n">
-        <v>0.125</v>
-      </c>
-    </row>
-    <row r="233">
-      <c r="A233" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B233" t="inlineStr">
-        <is>
-          <t>best</t>
-        </is>
-      </c>
-      <c r="C233" t="inlineStr">
-        <is>
-          <t>PTO_LA0</t>
-        </is>
-      </c>
-      <c r="D233" t="n">
-        <v>9</v>
-      </c>
-      <c r="E233" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F233" t="n">
-        <v>32</v>
-      </c>
-      <c r="G233" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="H233" t="n">
-        <v>0.2459346884189824</v>
-      </c>
-      <c r="I233" t="n">
-        <v>0.04347552147751577</v>
-      </c>
-      <c r="J233" t="n">
-        <v>0.1875</v>
-      </c>
-      <c r="K233" t="n">
-        <v>-0.125</v>
-      </c>
-    </row>
-    <row r="234">
-      <c r="A234" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B234" t="inlineStr">
-        <is>
-          <t>best</t>
-        </is>
-      </c>
-      <c r="C234" t="inlineStr">
-        <is>
-          <t>PTO_LA0</t>
-        </is>
-      </c>
-      <c r="D234" t="n">
-        <v>9</v>
-      </c>
-      <c r="E234" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F234" t="n">
-        <v>32</v>
-      </c>
-      <c r="G234" t="n">
-        <v>0.34375</v>
-      </c>
-      <c r="H234" t="n">
-        <v>0.4825587044348142</v>
-      </c>
-      <c r="I234" t="n">
-        <v>0.08530513305661301</v>
-      </c>
-      <c r="J234" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="K234" t="n">
-        <v>0.09375</v>
-      </c>
-    </row>
-    <row r="235">
-      <c r="A235" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B235" t="inlineStr">
-        <is>
-          <t>best</t>
-        </is>
-      </c>
-      <c r="C235" t="inlineStr">
-        <is>
-          <t>PTO_LA0</t>
-        </is>
-      </c>
-      <c r="D235" t="n">
-        <v>9</v>
-      </c>
-      <c r="E235" t="inlineStr">
-        <is>
-          <t>StartLowAndChangesToHigh</t>
-        </is>
-      </c>
-      <c r="F235" t="n">
-        <v>32</v>
-      </c>
-      <c r="G235" t="n">
-        <v>0.21875</v>
-      </c>
-      <c r="H235" t="n">
-        <v>0.4200134406451544</v>
-      </c>
-      <c r="I235" t="n">
-        <v>0.07424858801742054</v>
-      </c>
-      <c r="J235" t="n">
-        <v>0.1875</v>
-      </c>
-      <c r="K235" t="n">
-        <v>0.03125</v>
-      </c>
-    </row>
-    <row r="236">
-      <c r="A236" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B236" t="inlineStr">
-        <is>
-          <t>final</t>
-        </is>
-      </c>
-      <c r="C236" t="inlineStr">
-        <is>
-          <t>PTO_LA5</t>
-        </is>
-      </c>
-      <c r="D236" t="n">
-        <v>10</v>
-      </c>
-      <c r="E236" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F236" t="n">
-        <v>32</v>
-      </c>
-      <c r="G236" t="n">
-        <v>0.34375</v>
-      </c>
-      <c r="H236" t="n">
-        <v>0.4825587044348142</v>
-      </c>
-      <c r="I236" t="n">
-        <v>0.08530513305661301</v>
-      </c>
-      <c r="J236" t="n">
-        <v>0.1875</v>
-      </c>
-      <c r="K236" t="n">
-        <v>0.15625</v>
-      </c>
-    </row>
-    <row r="237">
-      <c r="A237" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B237" t="inlineStr">
-        <is>
-          <t>final</t>
-        </is>
-      </c>
-      <c r="C237" t="inlineStr">
-        <is>
-          <t>PTO_LA5</t>
-        </is>
-      </c>
-      <c r="D237" t="n">
-        <v>10</v>
-      </c>
-      <c r="E237" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F237" t="n">
-        <v>32</v>
-      </c>
-      <c r="G237" t="n">
-        <v>0.546875</v>
-      </c>
-      <c r="H237" t="n">
-        <v>0.4977266868861963</v>
-      </c>
-      <c r="I237" t="n">
-        <v>0.08798647886868571</v>
-      </c>
-      <c r="J237" t="n">
-        <v>0.203125</v>
-      </c>
-      <c r="K237" t="n">
-        <v>0.34375</v>
-      </c>
-    </row>
-    <row r="238">
-      <c r="A238" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B238" t="inlineStr">
-        <is>
-          <t>final</t>
-        </is>
-      </c>
-      <c r="C238" t="inlineStr">
-        <is>
-          <t>PTO_LA5</t>
-        </is>
-      </c>
-      <c r="D238" t="n">
-        <v>10</v>
-      </c>
-      <c r="E238" t="inlineStr">
-        <is>
-          <t>StartLowAndChangesToHigh</t>
-        </is>
-      </c>
-      <c r="F238" t="n">
-        <v>32</v>
-      </c>
-      <c r="G238" t="n">
-        <v>0.4375</v>
-      </c>
-      <c r="H238" t="n">
-        <v>0.5040161287741853</v>
-      </c>
-      <c r="I238" t="n">
-        <v>0.08909830562090465</v>
-      </c>
-      <c r="J238" t="n">
-        <v>0.175</v>
-      </c>
-      <c r="K238" t="n">
-        <v>0.2625</v>
-      </c>
-    </row>
-    <row r="239">
-      <c r="A239" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B239" t="inlineStr">
-        <is>
-          <t>best</t>
-        </is>
-      </c>
-      <c r="C239" t="inlineStr">
-        <is>
-          <t>PTO_LA5</t>
-        </is>
-      </c>
-      <c r="D239" t="n">
-        <v>7</v>
-      </c>
-      <c r="E239" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F239" t="n">
-        <v>32</v>
-      </c>
-      <c r="G239" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="H239" t="n">
-        <v>0.4918693768379647</v>
-      </c>
-      <c r="I239" t="n">
-        <v>0.08695104295503155</v>
-      </c>
-      <c r="J239" t="n">
-        <v>0.1875</v>
-      </c>
-      <c r="K239" t="n">
-        <v>0.1875</v>
-      </c>
-    </row>
-    <row r="240">
-      <c r="A240" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B240" t="inlineStr">
-        <is>
-          <t>best</t>
-        </is>
-      </c>
-      <c r="C240" t="inlineStr">
-        <is>
-          <t>PTO_LA5</t>
-        </is>
-      </c>
-      <c r="D240" t="n">
-        <v>7</v>
-      </c>
-      <c r="E240" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F240" t="n">
-        <v>32</v>
-      </c>
-      <c r="G240" t="n">
-        <v>0.265625</v>
-      </c>
-      <c r="H240" t="n">
-        <v>0.4396548316210592</v>
-      </c>
-      <c r="I240" t="n">
-        <v>0.07772072820517018</v>
-      </c>
-      <c r="J240" t="n">
-        <v>0.203125</v>
-      </c>
-      <c r="K240" t="n">
-        <v>0.0625</v>
-      </c>
-    </row>
-    <row r="241">
-      <c r="A241" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B241" t="inlineStr">
-        <is>
-          <t>best</t>
-        </is>
-      </c>
-      <c r="C241" t="inlineStr">
-        <is>
-          <t>PTO_LA5</t>
-        </is>
-      </c>
-      <c r="D241" t="n">
-        <v>7</v>
-      </c>
-      <c r="E241" t="inlineStr">
-        <is>
-          <t>StartLowAndChangesToHigh</t>
-        </is>
-      </c>
-      <c r="F241" t="n">
-        <v>32</v>
-      </c>
-      <c r="G241" t="n">
-        <v>0.15625</v>
-      </c>
-      <c r="H241" t="n">
-        <v>0.3689020326284735</v>
-      </c>
-      <c r="I241" t="n">
-        <v>0.06521328221627366</v>
-      </c>
-      <c r="J241" t="n">
-        <v>0.175</v>
-      </c>
-      <c r="K241" t="n">
-        <v>-0.01874999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -10805,7 +9773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K161"/>
+  <dimension ref="A1:K145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17057,694 +16025,6 @@
         <v>0.7034313725490198</v>
       </c>
     </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>final</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>GRPO_LA0</t>
-        </is>
-      </c>
-      <c r="D146" t="n">
-        <v>10</v>
-      </c>
-      <c r="E146" t="inlineStr">
-        <is>
-          <t>Obesity</t>
-        </is>
-      </c>
-      <c r="F146" t="n">
-        <v>48</v>
-      </c>
-      <c r="G146" t="n">
-        <v>0.1666666666666667</v>
-      </c>
-      <c r="H146" t="n">
-        <v>0.3766217885773548</v>
-      </c>
-      <c r="I146" t="n">
-        <v>0.05436067275445353</v>
-      </c>
-      <c r="J146" t="n">
-        <v>0.3150793650793651</v>
-      </c>
-      <c r="K146" t="n">
-        <v>-0.1484126984126984</v>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>final</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>GRPO_LA0</t>
-        </is>
-      </c>
-      <c r="D147" t="n">
-        <v>10</v>
-      </c>
-      <c r="E147" t="inlineStr">
-        <is>
-          <t>Smoking</t>
-        </is>
-      </c>
-      <c r="F147" t="n">
-        <v>48</v>
-      </c>
-      <c r="G147" t="n">
-        <v>0.1875</v>
-      </c>
-      <c r="H147" t="n">
-        <v>0.3944427796055833</v>
-      </c>
-      <c r="I147" t="n">
-        <v>0.05693291124629694</v>
-      </c>
-      <c r="J147" t="n">
-        <v>0.1666666666666667</v>
-      </c>
-      <c r="K147" t="n">
-        <v>0.02083333333333334</v>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>best</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>GRPO_LA0</t>
-        </is>
-      </c>
-      <c r="D148" t="n">
-        <v>3</v>
-      </c>
-      <c r="E148" t="inlineStr">
-        <is>
-          <t>Obesity</t>
-        </is>
-      </c>
-      <c r="F148" t="n">
-        <v>48</v>
-      </c>
-      <c r="G148" t="n">
-        <v>0.2986111111111111</v>
-      </c>
-      <c r="H148" t="n">
-        <v>0.4455696454031056</v>
-      </c>
-      <c r="I148" t="n">
-        <v>0.06431243867905229</v>
-      </c>
-      <c r="J148" t="n">
-        <v>0.3150793650793651</v>
-      </c>
-      <c r="K148" t="n">
-        <v>-0.01646825396825397</v>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>best</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>GRPO_LA0</t>
-        </is>
-      </c>
-      <c r="D149" t="n">
-        <v>3</v>
-      </c>
-      <c r="E149" t="inlineStr">
-        <is>
-          <t>Smoking</t>
-        </is>
-      </c>
-      <c r="F149" t="n">
-        <v>48</v>
-      </c>
-      <c r="G149" t="n">
-        <v>0.2708333333333333</v>
-      </c>
-      <c r="H149" t="n">
-        <v>0.4490928602896294</v>
-      </c>
-      <c r="I149" t="n">
-        <v>0.06482097094483914</v>
-      </c>
-      <c r="J149" t="n">
-        <v>0.1666666666666667</v>
-      </c>
-      <c r="K149" t="n">
-        <v>0.1041666666666667</v>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>final</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>GRPO_LA5</t>
-        </is>
-      </c>
-      <c r="D150" t="n">
-        <v>10</v>
-      </c>
-      <c r="E150" t="inlineStr">
-        <is>
-          <t>Obesity</t>
-        </is>
-      </c>
-      <c r="F150" t="n">
-        <v>48</v>
-      </c>
-      <c r="G150" t="n">
-        <v>0.8125</v>
-      </c>
-      <c r="H150" t="n">
-        <v>0.3944427796055833</v>
-      </c>
-      <c r="I150" t="n">
-        <v>0.05693291124629694</v>
-      </c>
-      <c r="J150" t="n">
-        <v>0.2597222222222222</v>
-      </c>
-      <c r="K150" t="n">
-        <v>0.5527777777777778</v>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>final</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>GRPO_LA5</t>
-        </is>
-      </c>
-      <c r="D151" t="n">
-        <v>10</v>
-      </c>
-      <c r="E151" t="inlineStr">
-        <is>
-          <t>Smoking</t>
-        </is>
-      </c>
-      <c r="F151" t="n">
-        <v>48</v>
-      </c>
-      <c r="G151" t="n">
-        <v>0.7916666666666666</v>
-      </c>
-      <c r="H151" t="n">
-        <v>0.4104140790860576</v>
-      </c>
-      <c r="I151" t="n">
-        <v>0.05923816975988693</v>
-      </c>
-      <c r="J151" t="n">
-        <v>0.1354166666666667</v>
-      </c>
-      <c r="K151" t="n">
-        <v>0.65625</v>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>best</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>GRPO_LA5</t>
-        </is>
-      </c>
-      <c r="D152" t="n">
-        <v>7</v>
-      </c>
-      <c r="E152" t="inlineStr">
-        <is>
-          <t>Obesity</t>
-        </is>
-      </c>
-      <c r="F152" t="n">
-        <v>48</v>
-      </c>
-      <c r="G152" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="H152" t="n">
-        <v>0.4892460547900817</v>
-      </c>
-      <c r="I152" t="n">
-        <v>0.07061658535825402</v>
-      </c>
-      <c r="J152" t="n">
-        <v>0.2597222222222222</v>
-      </c>
-      <c r="K152" t="n">
-        <v>0.3652777777777778</v>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>best</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>GRPO_LA5</t>
-        </is>
-      </c>
-      <c r="D153" t="n">
-        <v>7</v>
-      </c>
-      <c r="E153" t="inlineStr">
-        <is>
-          <t>Smoking</t>
-        </is>
-      </c>
-      <c r="F153" t="n">
-        <v>48</v>
-      </c>
-      <c r="G153" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="H153" t="n">
-        <v>0.4892460547900817</v>
-      </c>
-      <c r="I153" t="n">
-        <v>0.07061658535825402</v>
-      </c>
-      <c r="J153" t="n">
-        <v>0.1354166666666667</v>
-      </c>
-      <c r="K153" t="n">
-        <v>0.4895833333333334</v>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>final</t>
-        </is>
-      </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>PTO_LA0</t>
-        </is>
-      </c>
-      <c r="D154" t="n">
-        <v>10</v>
-      </c>
-      <c r="E154" t="inlineStr">
-        <is>
-          <t>Obesity</t>
-        </is>
-      </c>
-      <c r="F154" t="n">
-        <v>48</v>
-      </c>
-      <c r="G154" t="n">
-        <v>0.2291666666666667</v>
-      </c>
-      <c r="H154" t="n">
-        <v>0.4247443953937942</v>
-      </c>
-      <c r="I154" t="n">
-        <v>0.06130657275434798</v>
-      </c>
-      <c r="J154" t="n">
-        <v>0.1666666666666667</v>
-      </c>
-      <c r="K154" t="n">
-        <v>0.0625</v>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>final</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>PTO_LA0</t>
-        </is>
-      </c>
-      <c r="D155" t="n">
-        <v>10</v>
-      </c>
-      <c r="E155" t="inlineStr">
-        <is>
-          <t>Smoking</t>
-        </is>
-      </c>
-      <c r="F155" t="n">
-        <v>48</v>
-      </c>
-      <c r="G155" t="n">
-        <v>0.3020833333333333</v>
-      </c>
-      <c r="H155" t="n">
-        <v>0.4478161482131621</v>
-      </c>
-      <c r="I155" t="n">
-        <v>0.06463669342958263</v>
-      </c>
-      <c r="J155" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="K155" t="n">
-        <v>0.05208333333333331</v>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>best</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>PTO_LA0</t>
-        </is>
-      </c>
-      <c r="D156" t="n">
-        <v>9</v>
-      </c>
-      <c r="E156" t="inlineStr">
-        <is>
-          <t>Obesity</t>
-        </is>
-      </c>
-      <c r="F156" t="n">
-        <v>48</v>
-      </c>
-      <c r="G156" t="n">
-        <v>0.2083333333333333</v>
-      </c>
-      <c r="H156" t="n">
-        <v>0.4104140790860576</v>
-      </c>
-      <c r="I156" t="n">
-        <v>0.05923816975988693</v>
-      </c>
-      <c r="J156" t="n">
-        <v>0.1666666666666667</v>
-      </c>
-      <c r="K156" t="n">
-        <v>0.04166666666666669</v>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>best</t>
-        </is>
-      </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>PTO_LA0</t>
-        </is>
-      </c>
-      <c r="D157" t="n">
-        <v>9</v>
-      </c>
-      <c r="E157" t="inlineStr">
-        <is>
-          <t>Smoking</t>
-        </is>
-      </c>
-      <c r="F157" t="n">
-        <v>48</v>
-      </c>
-      <c r="G157" t="n">
-        <v>0.2083333333333333</v>
-      </c>
-      <c r="H157" t="n">
-        <v>0.4104140790860576</v>
-      </c>
-      <c r="I157" t="n">
-        <v>0.05923816975988693</v>
-      </c>
-      <c r="J157" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="K157" t="n">
-        <v>-0.04166666666666666</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>final</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>PTO_LA5</t>
-        </is>
-      </c>
-      <c r="D158" t="n">
-        <v>10</v>
-      </c>
-      <c r="E158" t="inlineStr">
-        <is>
-          <t>Obesity</t>
-        </is>
-      </c>
-      <c r="F158" t="n">
-        <v>48</v>
-      </c>
-      <c r="G158" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H158" t="n">
-        <v>0.5052911526399113</v>
-      </c>
-      <c r="I158" t="n">
-        <v>0.07293249574894728</v>
-      </c>
-      <c r="J158" t="n">
-        <v>0.1479166666666667</v>
-      </c>
-      <c r="K158" t="n">
-        <v>0.3520833333333333</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>final</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>PTO_LA5</t>
-        </is>
-      </c>
-      <c r="D159" t="n">
-        <v>10</v>
-      </c>
-      <c r="E159" t="inlineStr">
-        <is>
-          <t>Smoking</t>
-        </is>
-      </c>
-      <c r="F159" t="n">
-        <v>48</v>
-      </c>
-      <c r="G159" t="n">
-        <v>0.3854166666666667</v>
-      </c>
-      <c r="H159" t="n">
-        <v>0.4864065296197591</v>
-      </c>
-      <c r="I159" t="n">
-        <v>0.07020673520288989</v>
-      </c>
-      <c r="J159" t="n">
-        <v>0.2291666666666667</v>
-      </c>
-      <c r="K159" t="n">
-        <v>0.15625</v>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>best</t>
-        </is>
-      </c>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>PTO_LA5</t>
-        </is>
-      </c>
-      <c r="D160" t="n">
-        <v>7</v>
-      </c>
-      <c r="E160" t="inlineStr">
-        <is>
-          <t>Obesity</t>
-        </is>
-      </c>
-      <c r="F160" t="n">
-        <v>48</v>
-      </c>
-      <c r="G160" t="n">
-        <v>0.3645833333333333</v>
-      </c>
-      <c r="H160" t="n">
-        <v>0.480907645105136</v>
-      </c>
-      <c r="I160" t="n">
-        <v>0.06941303958919982</v>
-      </c>
-      <c r="J160" t="n">
-        <v>0.1479166666666667</v>
-      </c>
-      <c r="K160" t="n">
-        <v>0.2166666666666666</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>MIPROC</t>
-        </is>
-      </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>best</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>PTO_LA5</t>
-        </is>
-      </c>
-      <c r="D161" t="n">
-        <v>7</v>
-      </c>
-      <c r="E161" t="inlineStr">
-        <is>
-          <t>Smoking</t>
-        </is>
-      </c>
-      <c r="F161" t="n">
-        <v>48</v>
-      </c>
-      <c r="G161" t="n">
-        <v>0.1666666666666667</v>
-      </c>
-      <c r="H161" t="n">
-        <v>0.3766217885773547</v>
-      </c>
-      <c r="I161" t="n">
-        <v>0.05436067275445352</v>
-      </c>
-      <c r="J161" t="n">
-        <v>0.2291666666666667</v>
-      </c>
-      <c r="K161" t="n">
-        <v>-0.0625</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>